<commit_message>
back to old rule
</commit_message>
<xml_diff>
--- a/graphs/algorithms_time.xlsx
+++ b/graphs/algorithms_time.xlsx
@@ -473,12 +473,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-11-11 18:21:38</t>
+          <t>2025-11-18 14:22:53</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -492,27 +492,27 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>29</v>
+        <v>4638</v>
       </c>
       <c r="F2" t="n">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="G2" t="n">
-        <v>1.090450941002928</v>
+        <v>52.35931539512239</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0181741823500488</v>
+        <v>0.8726552565853732</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-11 18:21:40</t>
+          <t>2025-11-18 14:23:02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -526,27 +526,27 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>90</v>
+        <v>489</v>
       </c>
       <c r="F3" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="G3" t="n">
-        <v>1.877344737997191</v>
+        <v>8.190052408259362</v>
       </c>
       <c r="H3" t="n">
-        <v>0.03128907896661985</v>
+        <v>0.1365008734709894</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-11 18:21:50</t>
+          <t>2025-11-18 14:23:04</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -560,27 +560,27 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>495</v>
+        <v>90</v>
       </c>
       <c r="F4" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="G4" t="n">
-        <v>9.121524686001067</v>
+        <v>2.812568941153586</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1520254114333511</v>
+        <v>0.04687614901922643</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-11-11 18:23:01</t>
+          <t>2025-11-18 14:23:06</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -594,27 +594,27 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>4839</v>
+        <v>29</v>
       </c>
       <c r="F5" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="G5" t="n">
-        <v>69.20018173599965</v>
+        <v>1.448720317101106</v>
       </c>
       <c r="H5" t="n">
-        <v>1.153336362266661</v>
+        <v>0.02414533861835177</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-11-11 18:23:02</t>
+          <t>2025-11-18 14:23:54</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -628,27 +628,27 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>28</v>
+        <v>4168</v>
       </c>
       <c r="F6" t="n">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8799878770005307</v>
+        <v>47.49536211090162</v>
       </c>
       <c r="H6" t="n">
-        <v>0.01466646461667551</v>
+        <v>0.791589368515027</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-11 18:23:05</t>
+          <t>2025-11-18 14:24:02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -662,27 +662,27 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>89</v>
+        <v>468</v>
       </c>
       <c r="F7" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="G7" t="n">
-        <v>2.238453889000084</v>
+        <v>8.038439182098955</v>
       </c>
       <c r="H7" t="n">
-        <v>0.03730756481666807</v>
+        <v>0.1339739863683159</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-11-11 18:23:14</t>
+          <t>2025-11-18 14:24:05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -696,27 +696,27 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>496</v>
+        <v>87</v>
       </c>
       <c r="F8" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="G8" t="n">
-        <v>9.372370392000448</v>
+        <v>2.504834426101297</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1562061732000075</v>
+        <v>0.04174724043502162</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-11-11 18:24:30</t>
+          <t>2025-11-18 14:24:06</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -730,27 +730,27 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4801</v>
+        <v>28</v>
       </c>
       <c r="F9" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="G9" t="n">
-        <v>74.23086748700007</v>
+        <v>1.445969432126731</v>
       </c>
       <c r="H9" t="n">
-        <v>1.237181124783334</v>
+        <v>0.02409949053544551</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-11-11 18:24:32</t>
+          <t>2025-11-18 14:24:44</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -764,27 +764,27 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>21</v>
+        <v>3434</v>
       </c>
       <c r="F10" t="n">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="G10" t="n">
-        <v>0.7345539519992599</v>
+        <v>37.61558681307361</v>
       </c>
       <c r="H10" t="n">
-        <v>0.01224256586665433</v>
+        <v>0.6269264468845601</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-11-11 18:24:35</t>
+          <t>2025-11-18 14:24:50</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -798,27 +798,27 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>71</v>
+        <v>367</v>
       </c>
       <c r="F11" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="G11" t="n">
-        <v>2.821145431997138</v>
+        <v>5.797351956134662</v>
       </c>
       <c r="H11" t="n">
-        <v>0.04701909053328564</v>
+        <v>0.09662253260224436</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025-11-11 18:24:47</t>
+          <t>2025-11-18 14:24:52</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -832,27 +832,27 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>416</v>
+        <v>63</v>
       </c>
       <c r="F12" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="G12" t="n">
-        <v>12.2458623440034</v>
+        <v>1.977567512076348</v>
       </c>
       <c r="H12" t="n">
-        <v>0.20409770573339</v>
+        <v>0.0329594585346058</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2025-11-11 18:25:46</t>
+          <t>2025-11-18 14:24:54</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -866,27 +866,27 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>4312</v>
+        <v>21</v>
       </c>
       <c r="F13" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="G13" t="n">
-        <v>56.23307674700118</v>
+        <v>1.181469554081559</v>
       </c>
       <c r="H13" t="n">
-        <v>0.9372179457833529</v>
+        <v>0.01969115923469265</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-11-11 18:25:46</t>
+          <t>2025-11-18 14:25:28</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -900,27 +900,27 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>21</v>
+        <v>3156</v>
       </c>
       <c r="F14" t="n">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="G14" t="n">
-        <v>0.7074124360005953</v>
+        <v>33.60127035714686</v>
       </c>
       <c r="H14" t="n">
-        <v>0.01179020726667659</v>
+        <v>0.5600211726191143</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-11-11 18:25:48</t>
+          <t>2025-11-18 14:25:33</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -934,27 +934,27 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>61</v>
+        <v>298</v>
       </c>
       <c r="F15" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="G15" t="n">
-        <v>1.06148571200174</v>
+        <v>5.027003702241927</v>
       </c>
       <c r="H15" t="n">
-        <v>0.01769142853336234</v>
+        <v>0.08378339503736545</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-11-11 18:25:53</t>
+          <t>2025-11-18 14:25:35</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -968,27 +968,27 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>343</v>
+        <v>54</v>
       </c>
       <c r="F16" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="G16" t="n">
-        <v>5.037747738002508</v>
+        <v>1.729648160981014</v>
       </c>
       <c r="H16" t="n">
-        <v>0.08396246230004181</v>
+        <v>0.02882746934968357</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-11-11 18:26:38</t>
+          <t>2025-11-18 14:25:36</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1002,27 +1002,27 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>3906</v>
+        <v>21</v>
       </c>
       <c r="F17" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="G17" t="n">
-        <v>44.03667163800128</v>
+        <v>1.130774337099865</v>
       </c>
       <c r="H17" t="n">
-        <v>0.7339445273000214</v>
+        <v>0.01884623895166442</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-11-11 18:26:39</t>
+          <t>2025-11-18 14:26:17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1036,27 +1036,27 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>21</v>
+        <v>3740</v>
       </c>
       <c r="F18" t="n">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="G18" t="n">
-        <v>0.9112230270038708</v>
+        <v>40.83018840709701</v>
       </c>
       <c r="H18" t="n">
-        <v>0.01518705045006451</v>
+        <v>0.6805031401182835</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-11-11 18:26:43</t>
+          <t>2025-11-18 14:26:24</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1070,27 +1070,27 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>71</v>
+        <v>395</v>
       </c>
       <c r="F19" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="G19" t="n">
-        <v>2.630149836000783</v>
+        <v>6.570026815868914</v>
       </c>
       <c r="H19" t="n">
-        <v>0.04383583060001305</v>
+        <v>0.1095004469311486</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-11-11 18:26:50</t>
+          <t>2025-11-18 14:26:26</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1104,27 +1104,27 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>416</v>
+        <v>70</v>
       </c>
       <c r="F20" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="G20" t="n">
-        <v>7.165096169999742</v>
+        <v>2.0639825288672</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1194182694999957</v>
+        <v>0.03439970881445333</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-11-11 18:27:48</t>
+          <t>2025-11-18 14:26:27</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1138,27 +1138,27 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>4312</v>
+        <v>21</v>
       </c>
       <c r="F21" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="G21" t="n">
-        <v>55.94251504099884</v>
+        <v>1.197960330639035</v>
       </c>
       <c r="H21" t="n">
-        <v>0.9323752506833141</v>
+        <v>0.01996600551065058</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-11-11 18:27:49</t>
+          <t>2025-11-18 14:27:02</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1172,27 +1172,27 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>21</v>
+        <v>3108</v>
       </c>
       <c r="F22" t="n">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="G22" t="n">
-        <v>0.6933396990025358</v>
+        <v>34.16788941412233</v>
       </c>
       <c r="H22" t="n">
-        <v>0.01155566165004226</v>
+        <v>0.5694648235687054</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-11-11 18:27:51</t>
+          <t>2025-11-18 14:27:07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1206,27 +1206,27 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>61</v>
+        <v>300</v>
       </c>
       <c r="F23" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="G23" t="n">
-        <v>1.126936496999406</v>
+        <v>5.266137294936925</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0187822749499901</v>
+        <v>0.08776895491561541</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-11-11 18:27:56</t>
+          <t>2025-11-18 14:27:09</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1240,27 +1240,27 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>343</v>
+        <v>55</v>
       </c>
       <c r="F24" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="G24" t="n">
-        <v>5.419960380000703</v>
+        <v>1.735845480114222</v>
       </c>
       <c r="H24" t="n">
-        <v>0.09033267300001172</v>
+        <v>0.02893075800190369</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-11-11 18:28:44</t>
+          <t>2025-11-18 14:27:10</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1274,27 +1274,27 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>3906</v>
+        <v>21</v>
       </c>
       <c r="F25" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="G25" t="n">
-        <v>46.83515744800388</v>
+        <v>1.17214658879675</v>
       </c>
       <c r="H25" t="n">
-        <v>0.7805859574667314</v>
+        <v>0.01953577647994583</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2025-11-11 18:28:45</t>
+          <t>2025-11-18 14:27:56</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1308,27 +1308,27 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>21</v>
+        <v>4157</v>
       </c>
       <c r="F26" t="n">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="G26" t="n">
-        <v>0.474210974003654</v>
+        <v>45.30935580516234</v>
       </c>
       <c r="H26" t="n">
-        <v>0.007903516233394232</v>
+        <v>0.755155930086039</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2025-11-11 18:28:47</t>
+          <t>2025-11-18 14:28:03</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1342,27 +1342,27 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>71</v>
+        <v>412</v>
       </c>
       <c r="F27" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="G27" t="n">
-        <v>1.345441223998932</v>
+        <v>6.766640735790133</v>
       </c>
       <c r="H27" t="n">
-        <v>0.02242402039998221</v>
+        <v>0.1127773455965022</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-11-11 18:28:57</t>
+          <t>2025-11-18 14:28:05</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1376,27 +1376,27 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>416</v>
+        <v>71</v>
       </c>
       <c r="F28" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="G28" t="n">
-        <v>9.069889386995783</v>
+        <v>2.229082191130146</v>
       </c>
       <c r="H28" t="n">
-        <v>0.1511648231165964</v>
+        <v>0.03715136985216911</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-11-11 18:30:03</t>
+          <t>2025-11-18 14:28:06</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1410,27 +1410,27 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>4312</v>
+        <v>21</v>
       </c>
       <c r="F29" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="G29" t="n">
-        <v>64.39621659200202</v>
+        <v>1.153397918911651</v>
       </c>
       <c r="H29" t="n">
-        <v>1.073270276533367</v>
+        <v>0.01922329864852751</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-11-11 18:30:04</t>
+          <t>2025-11-18 14:28:58</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1444,27 +1444,27 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>28</v>
+        <v>4601</v>
       </c>
       <c r="F30" t="n">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="G30" t="n">
-        <v>0.8399279049990582</v>
+        <v>51.26599462004378</v>
       </c>
       <c r="H30" t="n">
-        <v>0.01399879841665097</v>
+        <v>0.8544332436673964</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2025-11-11 18:30:06</t>
+          <t>2025-11-18 14:29:07</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1478,27 +1478,27 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>89</v>
+        <v>490</v>
       </c>
       <c r="F31" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="G31" t="n">
-        <v>1.637787444000423</v>
+        <v>8.156948151998222</v>
       </c>
       <c r="H31" t="n">
-        <v>0.02729645740000706</v>
+        <v>0.135949135866637</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2025-11-11 18:30:16</t>
+          <t>2025-11-18 14:29:09</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1512,27 +1512,27 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>496</v>
+        <v>89</v>
       </c>
       <c r="F32" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="G32" t="n">
-        <v>10.13939006499641</v>
+        <v>2.586734340060502</v>
       </c>
       <c r="H32" t="n">
-        <v>0.1689898344166068</v>
+        <v>0.04311223900100837</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2025-11-11 18:31:45</t>
+          <t>2025-11-18 14:29:11</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1546,27 +1546,27 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>4801</v>
+        <v>28</v>
       </c>
       <c r="F33" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="G33" t="n">
-        <v>85.78955638800107</v>
+        <v>1.379107042914256</v>
       </c>
       <c r="H33" t="n">
-        <v>1.429825939800018</v>
+        <v>0.02298511738190427</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2025-11-11 18:31:46</t>
+          <t>2025-11-18 14:29:36</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1580,27 +1580,27 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>8</v>
+        <v>2286</v>
       </c>
       <c r="F34" t="n">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="G34" t="n">
-        <v>0.234185716999491</v>
+        <v>24.88865811517462</v>
       </c>
       <c r="H34" t="n">
-        <v>0.00390309528332485</v>
+        <v>0.4148109685862437</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2025-11-11 18:31:47</t>
+          <t>2025-11-18 14:29:39</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1614,27 +1614,27 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>42</v>
+        <v>176</v>
       </c>
       <c r="F35" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="G35" t="n">
-        <v>1.005994269999064</v>
+        <v>3.485725233098492</v>
       </c>
       <c r="H35" t="n">
-        <v>0.01676657116665107</v>
+        <v>0.05809542055164153</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2025-11-11 18:31:52</t>
+          <t>2025-11-18 14:29:41</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1648,27 +1648,27 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>194</v>
+        <v>42</v>
       </c>
       <c r="F36" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="G36" t="n">
-        <v>4.986561968002206</v>
+        <v>1.412741009145975</v>
       </c>
       <c r="H36" t="n">
-        <v>0.08310936613337011</v>
+        <v>0.02354568348576625</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2025-11-11 18:32:34</t>
+          <t>2025-11-18 14:29:42</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1682,27 +1682,27 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>2620</v>
+        <v>8</v>
       </c>
       <c r="F37" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="G37" t="n">
-        <v>40.28948705999937</v>
+        <v>0.6946657749358565</v>
       </c>
       <c r="H37" t="n">
-        <v>0.6714914509999895</v>
+        <v>0.01157776291559761</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2025-11-11 18:32:35</t>
+          <t>2025-11-18 14:30:26</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1716,27 +1716,27 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>29</v>
+        <v>3816</v>
       </c>
       <c r="F38" t="n">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="G38" t="n">
-        <v>1.061727988999337</v>
+        <v>43.61924562021159</v>
       </c>
       <c r="H38" t="n">
-        <v>0.01769546648332228</v>
+        <v>0.7269874270035265</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2025-11-11 18:32:37</t>
+          <t>2025-11-18 14:30:33</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1750,27 +1750,27 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>90</v>
+        <v>428</v>
       </c>
       <c r="F39" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="G39" t="n">
-        <v>2.107142629000009</v>
+        <v>7.342162705026567</v>
       </c>
       <c r="H39" t="n">
-        <v>0.03511904381666682</v>
+        <v>0.1223693784171094</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2025-11-11 18:32:49</t>
+          <t>2025-11-18 14:30:36</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1784,27 +1784,27 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>495</v>
+        <v>79</v>
       </c>
       <c r="F40" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="G40" t="n">
-        <v>10.57109351100371</v>
+        <v>2.554990296019241</v>
       </c>
       <c r="H40" t="n">
-        <v>0.1761848918500618</v>
+        <v>0.04258317160032069</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2025-11-11 18:34:04</t>
+          <t>2025-11-18 14:30:38</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Apriori</t>
+          <t>FPGrowth</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1819,19 +1819,19 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>4839</t>
+          <t>27</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>20000</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>72.85261867599911</v>
+        <v>1.499215939780697</v>
       </c>
       <c r="H41" t="n">
-        <v>1.214210311266652</v>
+        <v>0.02498693232967829</v>
       </c>
     </row>
   </sheetData>

</xml_diff>